<commit_message>
Per-part file links; offline spreadsheet variant
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/dataset.xlsx
+++ b/out/dataset.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z163"/>
+  <dimension ref="A1:AC163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -454,6 +454,9 @@
     <col width="14" customWidth="1" min="24" max="24"/>
     <col width="8" customWidth="1" min="25" max="25"/>
     <col width="20" customWidth="1" min="26" max="26"/>
+    <col width="20" customWidth="1" min="27" max="27"/>
+    <col width="20" customWidth="1" min="28" max="28"/>
+    <col width="20" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -584,6 +587,21 @@
       </c>
       <c r="Z1" s="1" t="inlineStr">
         <is>
+          <t>PDF folder</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>Markdown folder</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>Docx folder</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
           <t>Flags</t>
         </is>
       </c>
@@ -686,7 +704,22 @@
       <c r="Y2" t="n">
         <v>5</v>
       </c>
-      <c r="Z2" t="inlineStr"/>
+      <c r="Z2" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2026_616/</t>
+        </is>
+      </c>
+      <c r="AA2" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2026_616/</t>
+        </is>
+      </c>
+      <c r="AB2" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2026_616/</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -774,7 +807,22 @@
       <c r="Y3" t="n">
         <v>1</v>
       </c>
-      <c r="Z3" t="inlineStr"/>
+      <c r="Z3" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2026_580/</t>
+        </is>
+      </c>
+      <c r="AA3" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2026_580/</t>
+        </is>
+      </c>
+      <c r="AB3" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2026_580/</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -846,7 +894,22 @@
       <c r="Y4" t="n">
         <v>2</v>
       </c>
-      <c r="Z4" t="inlineStr"/>
+      <c r="Z4" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2026_570/</t>
+        </is>
+      </c>
+      <c r="AA4" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2026_570/</t>
+        </is>
+      </c>
+      <c r="AB4" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2026_570/</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -918,7 +981,22 @@
       <c r="Y5" t="n">
         <v>1</v>
       </c>
-      <c r="Z5" t="inlineStr"/>
+      <c r="Z5" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2026_565/</t>
+        </is>
+      </c>
+      <c r="AA5" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2026_565/</t>
+        </is>
+      </c>
+      <c r="AB5" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2026_565/</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -990,7 +1068,22 @@
       <c r="Y6" t="n">
         <v>1</v>
       </c>
-      <c r="Z6" t="inlineStr"/>
+      <c r="Z6" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2026_561/</t>
+        </is>
+      </c>
+      <c r="AA6" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2026_561/</t>
+        </is>
+      </c>
+      <c r="AB6" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2026_561/</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1062,7 +1155,22 @@
       <c r="Y7" t="n">
         <v>1</v>
       </c>
-      <c r="Z7" t="inlineStr"/>
+      <c r="Z7" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2026_165/</t>
+        </is>
+      </c>
+      <c r="AA7" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2026_165/</t>
+        </is>
+      </c>
+      <c r="AB7" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2026_165/</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1150,7 +1258,22 @@
       <c r="Y8" t="n">
         <v>3</v>
       </c>
-      <c r="Z8" t="inlineStr"/>
+      <c r="Z8" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2026_504/</t>
+        </is>
+      </c>
+      <c r="AA8" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2026_504/</t>
+        </is>
+      </c>
+      <c r="AB8" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2026_504/</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1242,7 +1365,22 @@
       <c r="Y9" t="n">
         <v>2</v>
       </c>
-      <c r="Z9" t="inlineStr"/>
+      <c r="Z9" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2026_502/</t>
+        </is>
+      </c>
+      <c r="AA9" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2026_502/</t>
+        </is>
+      </c>
+      <c r="AB9" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2026_502/</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1338,7 +1476,22 @@
       <c r="Y10" t="n">
         <v>1</v>
       </c>
-      <c r="Z10" t="inlineStr"/>
+      <c r="Z10" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2026_300/</t>
+        </is>
+      </c>
+      <c r="AA10" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2026_300/</t>
+        </is>
+      </c>
+      <c r="AB10" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2026_300/</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1430,7 +1583,22 @@
       <c r="Y11" t="n">
         <v>1</v>
       </c>
-      <c r="Z11" t="inlineStr"/>
+      <c r="Z11" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2026_114/</t>
+        </is>
+      </c>
+      <c r="AA11" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2026_114/</t>
+        </is>
+      </c>
+      <c r="AB11" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2026_114/</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1502,7 +1670,22 @@
       <c r="Y12" t="n">
         <v>3</v>
       </c>
-      <c r="Z12" t="inlineStr"/>
+      <c r="Z12" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2026_321/</t>
+        </is>
+      </c>
+      <c r="AA12" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2026_321/</t>
+        </is>
+      </c>
+      <c r="AB12" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2026_321/</t>
+        </is>
+      </c>
+      <c r="AC12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1598,7 +1781,22 @@
       <c r="Y13" t="n">
         <v>1</v>
       </c>
-      <c r="Z13" t="inlineStr"/>
+      <c r="Z13" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2026_89/</t>
+        </is>
+      </c>
+      <c r="AA13" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2026_89/</t>
+        </is>
+      </c>
+      <c r="AB13" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2026_89/</t>
+        </is>
+      </c>
+      <c r="AC13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1690,7 +1888,22 @@
       <c r="Y14" t="n">
         <v>1</v>
       </c>
-      <c r="Z14" t="inlineStr"/>
+      <c r="Z14" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2026_71/</t>
+        </is>
+      </c>
+      <c r="AA14" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2026_71/</t>
+        </is>
+      </c>
+      <c r="AB14" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2026_71/</t>
+        </is>
+      </c>
+      <c r="AC14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1762,7 +1975,22 @@
       <c r="Y15" t="n">
         <v>1</v>
       </c>
-      <c r="Z15" t="inlineStr"/>
+      <c r="Z15" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2026_102/</t>
+        </is>
+      </c>
+      <c r="AA15" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2026_102/</t>
+        </is>
+      </c>
+      <c r="AB15" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2026_102/</t>
+        </is>
+      </c>
+      <c r="AC15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1834,7 +2062,22 @@
       <c r="Y16" t="n">
         <v>3</v>
       </c>
-      <c r="Z16" t="inlineStr"/>
+      <c r="Z16" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2026_13/</t>
+        </is>
+      </c>
+      <c r="AA16" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2026_13/</t>
+        </is>
+      </c>
+      <c r="AB16" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2026_13/</t>
+        </is>
+      </c>
+      <c r="AC16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1930,7 +2173,22 @@
       <c r="Y17" t="n">
         <v>1</v>
       </c>
-      <c r="Z17" t="inlineStr"/>
+      <c r="Z17" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2026_11/</t>
+        </is>
+      </c>
+      <c r="AA17" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2026_11/</t>
+        </is>
+      </c>
+      <c r="AB17" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2026_11/</t>
+        </is>
+      </c>
+      <c r="AC17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2026,7 +2284,22 @@
       <c r="Y18" t="n">
         <v>2</v>
       </c>
-      <c r="Z18" t="inlineStr"/>
+      <c r="Z18" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2025_988/</t>
+        </is>
+      </c>
+      <c r="AA18" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2025_988/</t>
+        </is>
+      </c>
+      <c r="AB18" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2025_988/</t>
+        </is>
+      </c>
+      <c r="AC18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2122,7 +2395,22 @@
       <c r="Y19" t="n">
         <v>1</v>
       </c>
-      <c r="Z19" t="inlineStr"/>
+      <c r="Z19" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2025_1060/</t>
+        </is>
+      </c>
+      <c r="AA19" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2025_1060/</t>
+        </is>
+      </c>
+      <c r="AB19" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2025_1060/</t>
+        </is>
+      </c>
+      <c r="AC19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2222,7 +2510,22 @@
       <c r="Y20" t="n">
         <v>2</v>
       </c>
-      <c r="Z20" t="inlineStr"/>
+      <c r="Z20" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2025_1058/</t>
+        </is>
+      </c>
+      <c r="AA20" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2025_1058/</t>
+        </is>
+      </c>
+      <c r="AB20" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2025_1058/</t>
+        </is>
+      </c>
+      <c r="AC20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2294,7 +2597,22 @@
       <c r="Y21" t="n">
         <v>1</v>
       </c>
-      <c r="Z21" t="inlineStr"/>
+      <c r="Z21" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2025_2000/</t>
+        </is>
+      </c>
+      <c r="AA21" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2025_2000/</t>
+        </is>
+      </c>
+      <c r="AB21" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2025_2000/</t>
+        </is>
+      </c>
+      <c r="AC21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2366,7 +2684,22 @@
       <c r="Y22" t="n">
         <v>1</v>
       </c>
-      <c r="Z22" t="inlineStr"/>
+      <c r="Z22" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2025_943/</t>
+        </is>
+      </c>
+      <c r="AA22" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2025_943/</t>
+        </is>
+      </c>
+      <c r="AB22" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2025_943/</t>
+        </is>
+      </c>
+      <c r="AC22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2438,7 +2771,22 @@
       <c r="Y23" t="n">
         <v>2</v>
       </c>
-      <c r="Z23" t="inlineStr"/>
+      <c r="Z23" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2025_398/</t>
+        </is>
+      </c>
+      <c r="AA23" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2025_398/</t>
+        </is>
+      </c>
+      <c r="AB23" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2025_398/</t>
+        </is>
+      </c>
+      <c r="AC23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2526,7 +2874,22 @@
       <c r="Y24" t="n">
         <v>1</v>
       </c>
-      <c r="Z24" t="inlineStr"/>
+      <c r="Z24" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2025_838/</t>
+        </is>
+      </c>
+      <c r="AA24" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2025_838/</t>
+        </is>
+      </c>
+      <c r="AB24" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2025_838/</t>
+        </is>
+      </c>
+      <c r="AC24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2598,7 +2961,22 @@
       <c r="Y25" t="n">
         <v>1</v>
       </c>
-      <c r="Z25" t="inlineStr">
+      <c r="Z25" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2025_288/</t>
+        </is>
+      </c>
+      <c r="AA25" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2025_288/</t>
+        </is>
+      </c>
+      <c r="AB25" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2025_288/</t>
+        </is>
+      </c>
+      <c r="AC25" t="inlineStr">
         <is>
           <t>download_failed_part1</t>
         </is>
@@ -2698,7 +3076,22 @@
       <c r="Y26" t="n">
         <v>1</v>
       </c>
-      <c r="Z26" t="inlineStr"/>
+      <c r="Z26" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2025_592/</t>
+        </is>
+      </c>
+      <c r="AA26" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2025_592/</t>
+        </is>
+      </c>
+      <c r="AB26" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2025_592/</t>
+        </is>
+      </c>
+      <c r="AC26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2770,7 +3163,22 @@
       <c r="Y27" t="n">
         <v>1</v>
       </c>
-      <c r="Z27" t="inlineStr"/>
+      <c r="Z27" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2025_232/</t>
+        </is>
+      </c>
+      <c r="AA27" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2025_232/</t>
+        </is>
+      </c>
+      <c r="AB27" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2025_232/</t>
+        </is>
+      </c>
+      <c r="AC27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2866,7 +3274,22 @@
       <c r="Y28" t="n">
         <v>1</v>
       </c>
-      <c r="Z28" t="inlineStr"/>
+      <c r="Z28" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2025_192/</t>
+        </is>
+      </c>
+      <c r="AA28" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2025_192/</t>
+        </is>
+      </c>
+      <c r="AB28" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2025_192/</t>
+        </is>
+      </c>
+      <c r="AC28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2938,7 +3361,22 @@
       <c r="Y29" t="n">
         <v>1</v>
       </c>
-      <c r="Z29" t="inlineStr"/>
+      <c r="Z29" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2025_590/</t>
+        </is>
+      </c>
+      <c r="AA29" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2025_590/</t>
+        </is>
+      </c>
+      <c r="AB29" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2025_590/</t>
+        </is>
+      </c>
+      <c r="AC29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -3010,7 +3448,22 @@
       <c r="Y30" t="n">
         <v>1</v>
       </c>
-      <c r="Z30" t="inlineStr"/>
+      <c r="Z30" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2025_565/</t>
+        </is>
+      </c>
+      <c r="AA30" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2025_565/</t>
+        </is>
+      </c>
+      <c r="AB30" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2025_565/</t>
+        </is>
+      </c>
+      <c r="AC30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -3082,7 +3535,22 @@
       <c r="Y31" t="n">
         <v>1</v>
       </c>
-      <c r="Z31" t="inlineStr"/>
+      <c r="Z31" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2025_560/</t>
+        </is>
+      </c>
+      <c r="AA31" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2025_560/</t>
+        </is>
+      </c>
+      <c r="AB31" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2025_560/</t>
+        </is>
+      </c>
+      <c r="AC31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -3174,7 +3642,22 @@
       <c r="Y32" t="n">
         <v>1</v>
       </c>
-      <c r="Z32" t="inlineStr"/>
+      <c r="Z32" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2025_555/</t>
+        </is>
+      </c>
+      <c r="AA32" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2025_555/</t>
+        </is>
+      </c>
+      <c r="AB32" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2025_555/</t>
+        </is>
+      </c>
+      <c r="AC32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -3262,7 +3745,22 @@
       <c r="Y33" t="n">
         <v>1</v>
       </c>
-      <c r="Z33" t="inlineStr"/>
+      <c r="Z33" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2025_552/</t>
+        </is>
+      </c>
+      <c r="AA33" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2025_552/</t>
+        </is>
+      </c>
+      <c r="AB33" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2025_552/</t>
+        </is>
+      </c>
+      <c r="AC33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -3358,7 +3856,22 @@
       <c r="Y34" t="n">
         <v>1</v>
       </c>
-      <c r="Z34" t="inlineStr"/>
+      <c r="Z34" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2025_550/</t>
+        </is>
+      </c>
+      <c r="AA34" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2025_550/</t>
+        </is>
+      </c>
+      <c r="AB34" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2025_550/</t>
+        </is>
+      </c>
+      <c r="AC34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -3450,7 +3963,22 @@
       <c r="Y35" t="n">
         <v>1</v>
       </c>
-      <c r="Z35" t="inlineStr"/>
+      <c r="Z35" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2025_545/</t>
+        </is>
+      </c>
+      <c r="AA35" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2025_545/</t>
+        </is>
+      </c>
+      <c r="AB35" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2025_545/</t>
+        </is>
+      </c>
+      <c r="AC35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -3542,7 +4070,22 @@
       <c r="Y36" t="n">
         <v>2</v>
       </c>
-      <c r="Z36" t="inlineStr"/>
+      <c r="Z36" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2025_335/</t>
+        </is>
+      </c>
+      <c r="AA36" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2025_335/</t>
+        </is>
+      </c>
+      <c r="AB36" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2025_335/</t>
+        </is>
+      </c>
+      <c r="AC36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -3614,7 +4157,22 @@
       <c r="Y37" t="n">
         <v>1</v>
       </c>
-      <c r="Z37" t="inlineStr"/>
+      <c r="Z37" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2025_825/</t>
+        </is>
+      </c>
+      <c r="AA37" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2025_825/</t>
+        </is>
+      </c>
+      <c r="AB37" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2025_825/</t>
+        </is>
+      </c>
+      <c r="AC37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -3714,7 +4272,22 @@
       <c r="Y38" t="n">
         <v>1</v>
       </c>
-      <c r="Z38" t="inlineStr"/>
+      <c r="Z38" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2025_96/</t>
+        </is>
+      </c>
+      <c r="AA38" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2025_96/</t>
+        </is>
+      </c>
+      <c r="AB38" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2025_96/</t>
+        </is>
+      </c>
+      <c r="AC38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -3786,7 +4359,22 @@
       <c r="Y39" t="n">
         <v>1</v>
       </c>
-      <c r="Z39" t="inlineStr">
+      <c r="Z39" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2024_155/</t>
+        </is>
+      </c>
+      <c r="AA39" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2024_155/</t>
+        </is>
+      </c>
+      <c r="AB39" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2024_155/</t>
+        </is>
+      </c>
+      <c r="AC39" t="inlineStr">
         <is>
           <t>download_failed_part1</t>
         </is>
@@ -3862,7 +4450,22 @@
       <c r="Y40" t="n">
         <v>1</v>
       </c>
-      <c r="Z40" t="inlineStr"/>
+      <c r="Z40" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2024_62/</t>
+        </is>
+      </c>
+      <c r="AA40" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2024_62/</t>
+        </is>
+      </c>
+      <c r="AB40" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2024_62/</t>
+        </is>
+      </c>
+      <c r="AC40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3962,7 +4565,22 @@
       <c r="Y41" t="n">
         <v>2</v>
       </c>
-      <c r="Z41" t="inlineStr"/>
+      <c r="Z41" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2024_67/</t>
+        </is>
+      </c>
+      <c r="AA41" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2024_67/</t>
+        </is>
+      </c>
+      <c r="AB41" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2024_67/</t>
+        </is>
+      </c>
+      <c r="AC41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -4054,7 +4672,22 @@
       <c r="Y42" t="n">
         <v>5</v>
       </c>
-      <c r="Z42" t="inlineStr"/>
+      <c r="Z42" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2024_63/</t>
+        </is>
+      </c>
+      <c r="AA42" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2024_63/</t>
+        </is>
+      </c>
+      <c r="AB42" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2024_63/</t>
+        </is>
+      </c>
+      <c r="AC42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -4126,7 +4759,22 @@
       <c r="Y43" t="n">
         <v>1</v>
       </c>
-      <c r="Z43" t="inlineStr"/>
+      <c r="Z43" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2024_33/</t>
+        </is>
+      </c>
+      <c r="AA43" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2024_33/</t>
+        </is>
+      </c>
+      <c r="AB43" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2024_33/</t>
+        </is>
+      </c>
+      <c r="AC43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -4226,7 +4874,22 @@
       <c r="Y44" t="n">
         <v>1</v>
       </c>
-      <c r="Z44" t="inlineStr"/>
+      <c r="Z44" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2024_15/</t>
+        </is>
+      </c>
+      <c r="AA44" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2024_15/</t>
+        </is>
+      </c>
+      <c r="AB44" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2024_15/</t>
+        </is>
+      </c>
+      <c r="AC44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -4298,7 +4961,22 @@
       <c r="Y45" t="n">
         <v>1</v>
       </c>
-      <c r="Z45" t="inlineStr"/>
+      <c r="Z45" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2024_10/</t>
+        </is>
+      </c>
+      <c r="AA45" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2024_10/</t>
+        </is>
+      </c>
+      <c r="AB45" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2024_10/</t>
+        </is>
+      </c>
+      <c r="AC45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -4397,7 +5075,22 @@
       <c r="Y46" t="n">
         <v>1</v>
       </c>
-      <c r="Z46" t="inlineStr"/>
+      <c r="Z46" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_663/</t>
+        </is>
+      </c>
+      <c r="AA46" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_663/</t>
+        </is>
+      </c>
+      <c r="AB46" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_663/</t>
+        </is>
+      </c>
+      <c r="AC46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -4469,7 +5162,22 @@
       <c r="Y47" t="n">
         <v>2</v>
       </c>
-      <c r="Z47" t="inlineStr"/>
+      <c r="Z47" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_401/</t>
+        </is>
+      </c>
+      <c r="AA47" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_401/</t>
+        </is>
+      </c>
+      <c r="AB47" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_401/</t>
+        </is>
+      </c>
+      <c r="AC47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -4569,7 +5277,22 @@
       <c r="Y48" t="n">
         <v>1</v>
       </c>
-      <c r="Z48" t="inlineStr"/>
+      <c r="Z48" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_941/</t>
+        </is>
+      </c>
+      <c r="AA48" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_941/</t>
+        </is>
+      </c>
+      <c r="AB48" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_941/</t>
+        </is>
+      </c>
+      <c r="AC48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -4641,7 +5364,22 @@
       <c r="Y49" t="n">
         <v>1</v>
       </c>
-      <c r="Z49" t="inlineStr"/>
+      <c r="Z49" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_906/</t>
+        </is>
+      </c>
+      <c r="AA49" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_906/</t>
+        </is>
+      </c>
+      <c r="AB49" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_906/</t>
+        </is>
+      </c>
+      <c r="AC49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -4737,7 +5475,22 @@
       <c r="Y50" t="n">
         <v>1</v>
       </c>
-      <c r="Z50" t="inlineStr"/>
+      <c r="Z50" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_386/</t>
+        </is>
+      </c>
+      <c r="AA50" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_386/</t>
+        </is>
+      </c>
+      <c r="AB50" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_386/</t>
+        </is>
+      </c>
+      <c r="AC50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -4837,7 +5590,22 @@
       <c r="Y51" t="n">
         <v>1</v>
       </c>
-      <c r="Z51" t="inlineStr"/>
+      <c r="Z51" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_373/</t>
+        </is>
+      </c>
+      <c r="AA51" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_373/</t>
+        </is>
+      </c>
+      <c r="AB51" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_373/</t>
+        </is>
+      </c>
+      <c r="AC51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -4937,7 +5705,22 @@
       <c r="Y52" t="n">
         <v>1</v>
       </c>
-      <c r="Z52" t="inlineStr"/>
+      <c r="Z52" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_717/</t>
+        </is>
+      </c>
+      <c r="AA52" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_717/</t>
+        </is>
+      </c>
+      <c r="AB52" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_717/</t>
+        </is>
+      </c>
+      <c r="AC52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -5033,7 +5816,22 @@
       <c r="Y53" t="n">
         <v>1</v>
       </c>
-      <c r="Z53" t="inlineStr"/>
+      <c r="Z53" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_351/</t>
+        </is>
+      </c>
+      <c r="AA53" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_351/</t>
+        </is>
+      </c>
+      <c r="AB53" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_351/</t>
+        </is>
+      </c>
+      <c r="AC53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -5105,7 +5903,22 @@
       <c r="Y54" t="n">
         <v>2</v>
       </c>
-      <c r="Z54" t="inlineStr"/>
+      <c r="Z54" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_335/</t>
+        </is>
+      </c>
+      <c r="AA54" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_335/</t>
+        </is>
+      </c>
+      <c r="AB54" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_335/</t>
+        </is>
+      </c>
+      <c r="AC54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -5177,7 +5990,22 @@
       <c r="Y55" t="n">
         <v>3</v>
       </c>
-      <c r="Z55" t="inlineStr"/>
+      <c r="Z55" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_332/</t>
+        </is>
+      </c>
+      <c r="AA55" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_332/</t>
+        </is>
+      </c>
+      <c r="AB55" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_332/</t>
+        </is>
+      </c>
+      <c r="AC55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -5269,7 +6097,22 @@
       <c r="Y56" t="n">
         <v>1</v>
       </c>
-      <c r="Z56" t="inlineStr"/>
+      <c r="Z56" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_314/</t>
+        </is>
+      </c>
+      <c r="AA56" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_314/</t>
+        </is>
+      </c>
+      <c r="AB56" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_314/</t>
+        </is>
+      </c>
+      <c r="AC56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -5342,7 +6185,22 @@
       <c r="Y57" t="n">
         <v>1</v>
       </c>
-      <c r="Z57" t="inlineStr"/>
+      <c r="Z57" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_302/</t>
+        </is>
+      </c>
+      <c r="AA57" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_302/</t>
+        </is>
+      </c>
+      <c r="AB57" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_302/</t>
+        </is>
+      </c>
+      <c r="AC57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -5414,7 +6272,22 @@
       <c r="Y58" t="n">
         <v>1</v>
       </c>
-      <c r="Z58" t="inlineStr"/>
+      <c r="Z58" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_290/</t>
+        </is>
+      </c>
+      <c r="AA58" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_290/</t>
+        </is>
+      </c>
+      <c r="AB58" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_290/</t>
+        </is>
+      </c>
+      <c r="AC58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -5510,7 +6383,22 @@
       <c r="Y59" t="n">
         <v>2</v>
       </c>
-      <c r="Z59" t="inlineStr"/>
+      <c r="Z59" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_293/</t>
+        </is>
+      </c>
+      <c r="AA59" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_293/</t>
+        </is>
+      </c>
+      <c r="AB59" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_293/</t>
+        </is>
+      </c>
+      <c r="AC59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -5606,7 +6494,22 @@
       <c r="Y60" t="n">
         <v>1</v>
       </c>
-      <c r="Z60" t="inlineStr"/>
+      <c r="Z60" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_269/</t>
+        </is>
+      </c>
+      <c r="AA60" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_269/</t>
+        </is>
+      </c>
+      <c r="AB60" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_269/</t>
+        </is>
+      </c>
+      <c r="AC60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -5678,7 +6581,22 @@
       <c r="Y61" t="n">
         <v>1</v>
       </c>
-      <c r="Z61" t="inlineStr"/>
+      <c r="Z61" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_265/</t>
+        </is>
+      </c>
+      <c r="AA61" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_265/</t>
+        </is>
+      </c>
+      <c r="AB61" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_265/</t>
+        </is>
+      </c>
+      <c r="AC61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -5750,7 +6668,22 @@
       <c r="Y62" t="n">
         <v>1</v>
       </c>
-      <c r="Z62" t="inlineStr"/>
+      <c r="Z62" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_396/</t>
+        </is>
+      </c>
+      <c r="AA62" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_396/</t>
+        </is>
+      </c>
+      <c r="AB62" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_396/</t>
+        </is>
+      </c>
+      <c r="AC62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -5846,7 +6779,22 @@
       <c r="Y63" t="n">
         <v>4</v>
       </c>
-      <c r="Z63" t="inlineStr"/>
+      <c r="Z63" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_256/</t>
+        </is>
+      </c>
+      <c r="AA63" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_256/</t>
+        </is>
+      </c>
+      <c r="AB63" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_256/</t>
+        </is>
+      </c>
+      <c r="AC63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -5923,7 +6871,22 @@
       <c r="Y64" t="n">
         <v>1</v>
       </c>
-      <c r="Z64" t="inlineStr"/>
+      <c r="Z64" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_252/</t>
+        </is>
+      </c>
+      <c r="AA64" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_252/</t>
+        </is>
+      </c>
+      <c r="AB64" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_252/</t>
+        </is>
+      </c>
+      <c r="AC64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -5995,7 +6958,22 @@
       <c r="Y65" t="n">
         <v>1</v>
       </c>
-      <c r="Z65" t="inlineStr"/>
+      <c r="Z65" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_246/</t>
+        </is>
+      </c>
+      <c r="AA65" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_246/</t>
+        </is>
+      </c>
+      <c r="AB65" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_246/</t>
+        </is>
+      </c>
+      <c r="AC65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -6091,7 +7069,22 @@
       <c r="Y66" t="n">
         <v>1</v>
       </c>
-      <c r="Z66" t="inlineStr"/>
+      <c r="Z66" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_445/</t>
+        </is>
+      </c>
+      <c r="AA66" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_445/</t>
+        </is>
+      </c>
+      <c r="AB66" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_445/</t>
+        </is>
+      </c>
+      <c r="AC66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -6187,7 +7180,22 @@
       <c r="Y67" t="n">
         <v>1</v>
       </c>
-      <c r="Z67" t="inlineStr"/>
+      <c r="Z67" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_443/</t>
+        </is>
+      </c>
+      <c r="AA67" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_443/</t>
+        </is>
+      </c>
+      <c r="AB67" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_443/</t>
+        </is>
+      </c>
+      <c r="AC67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -6287,7 +7295,22 @@
       <c r="Y68" t="n">
         <v>1</v>
       </c>
-      <c r="Z68" t="inlineStr"/>
+      <c r="Z68" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_441/</t>
+        </is>
+      </c>
+      <c r="AA68" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_441/</t>
+        </is>
+      </c>
+      <c r="AB68" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_441/</t>
+        </is>
+      </c>
+      <c r="AC68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -6359,7 +7382,22 @@
       <c r="Y69" t="n">
         <v>1</v>
       </c>
-      <c r="Z69" t="inlineStr"/>
+      <c r="Z69" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_240/</t>
+        </is>
+      </c>
+      <c r="AA69" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_240/</t>
+        </is>
+      </c>
+      <c r="AB69" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_240/</t>
+        </is>
+      </c>
+      <c r="AC69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -6451,7 +7489,22 @@
       <c r="Y70" t="n">
         <v>4</v>
       </c>
-      <c r="Z70" t="inlineStr"/>
+      <c r="Z70" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_421/</t>
+        </is>
+      </c>
+      <c r="AA70" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_421/</t>
+        </is>
+      </c>
+      <c r="AB70" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_421/</t>
+        </is>
+      </c>
+      <c r="AC70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -6539,7 +7592,22 @@
       <c r="Y71" t="n">
         <v>5</v>
       </c>
-      <c r="Z71" t="inlineStr"/>
+      <c r="Z71" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_417/</t>
+        </is>
+      </c>
+      <c r="AA71" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_417/</t>
+        </is>
+      </c>
+      <c r="AB71" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_417/</t>
+        </is>
+      </c>
+      <c r="AC71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -6614,7 +7682,22 @@
       <c r="Y72" t="n">
         <v>1</v>
       </c>
-      <c r="Z72" t="inlineStr"/>
+      <c r="Z72" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_414/</t>
+        </is>
+      </c>
+      <c r="AA72" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_414/</t>
+        </is>
+      </c>
+      <c r="AB72" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_414/</t>
+        </is>
+      </c>
+      <c r="AC72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -6714,7 +7797,22 @@
       <c r="Y73" t="n">
         <v>1</v>
       </c>
-      <c r="Z73" t="inlineStr"/>
+      <c r="Z73" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_412/</t>
+        </is>
+      </c>
+      <c r="AA73" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_412/</t>
+        </is>
+      </c>
+      <c r="AB73" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_412/</t>
+        </is>
+      </c>
+      <c r="AC73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -6786,7 +7884,22 @@
       <c r="Y74" t="n">
         <v>1</v>
       </c>
-      <c r="Z74" t="inlineStr"/>
+      <c r="Z74" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_233/</t>
+        </is>
+      </c>
+      <c r="AA74" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_233/</t>
+        </is>
+      </c>
+      <c r="AB74" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_233/</t>
+        </is>
+      </c>
+      <c r="AC74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -6858,7 +7971,22 @@
       <c r="Y75" t="n">
         <v>1</v>
       </c>
-      <c r="Z75" t="inlineStr"/>
+      <c r="Z75" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_231/</t>
+        </is>
+      </c>
+      <c r="AA75" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_231/</t>
+        </is>
+      </c>
+      <c r="AB75" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_231/</t>
+        </is>
+      </c>
+      <c r="AC75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -6930,7 +8058,22 @@
       <c r="Y76" t="n">
         <v>1</v>
       </c>
-      <c r="Z76" t="inlineStr"/>
+      <c r="Z76" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_224/</t>
+        </is>
+      </c>
+      <c r="AA76" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_224/</t>
+        </is>
+      </c>
+      <c r="AB76" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_224/</t>
+        </is>
+      </c>
+      <c r="AC76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -7002,7 +8145,22 @@
       <c r="Y77" t="n">
         <v>1</v>
       </c>
-      <c r="Z77" t="inlineStr"/>
+      <c r="Z77" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_216/</t>
+        </is>
+      </c>
+      <c r="AA77" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_216/</t>
+        </is>
+      </c>
+      <c r="AB77" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_216/</t>
+        </is>
+      </c>
+      <c r="AC77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -7077,7 +8235,22 @@
       <c r="Y78" t="n">
         <v>7</v>
       </c>
-      <c r="Z78" t="inlineStr"/>
+      <c r="Z78" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_101/</t>
+        </is>
+      </c>
+      <c r="AA78" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_101/</t>
+        </is>
+      </c>
+      <c r="AB78" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_101/</t>
+        </is>
+      </c>
+      <c r="AC78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -7165,7 +8338,22 @@
       <c r="Y79" t="n">
         <v>1</v>
       </c>
-      <c r="Z79" t="inlineStr"/>
+      <c r="Z79" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_204/</t>
+        </is>
+      </c>
+      <c r="AA79" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_204/</t>
+        </is>
+      </c>
+      <c r="AB79" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_204/</t>
+        </is>
+      </c>
+      <c r="AC79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -7238,7 +8426,22 @@
       <c r="Y80" t="n">
         <v>1</v>
       </c>
-      <c r="Z80" t="inlineStr"/>
+      <c r="Z80" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_167/</t>
+        </is>
+      </c>
+      <c r="AA80" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_167/</t>
+        </is>
+      </c>
+      <c r="AB80" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_167/</t>
+        </is>
+      </c>
+      <c r="AC80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -7334,7 +8537,22 @@
       <c r="Y81" t="n">
         <v>1</v>
       </c>
-      <c r="Z81" t="inlineStr"/>
+      <c r="Z81" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_165/</t>
+        </is>
+      </c>
+      <c r="AA81" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_165/</t>
+        </is>
+      </c>
+      <c r="AB81" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_165/</t>
+        </is>
+      </c>
+      <c r="AC81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -7434,7 +8652,22 @@
       <c r="Y82" t="n">
         <v>2</v>
       </c>
-      <c r="Z82" t="inlineStr"/>
+      <c r="Z82" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_159/</t>
+        </is>
+      </c>
+      <c r="AA82" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_159/</t>
+        </is>
+      </c>
+      <c r="AB82" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_159/</t>
+        </is>
+      </c>
+      <c r="AC82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -7506,7 +8739,22 @@
       <c r="Y83" t="n">
         <v>1</v>
       </c>
-      <c r="Z83" t="inlineStr"/>
+      <c r="Z83" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_148/</t>
+        </is>
+      </c>
+      <c r="AA83" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_148/</t>
+        </is>
+      </c>
+      <c r="AB83" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_148/</t>
+        </is>
+      </c>
+      <c r="AC83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -7578,7 +8826,22 @@
       <c r="Y84" t="n">
         <v>1</v>
       </c>
-      <c r="Z84" t="inlineStr"/>
+      <c r="Z84" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_145/</t>
+        </is>
+      </c>
+      <c r="AA84" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_145/</t>
+        </is>
+      </c>
+      <c r="AB84" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_145/</t>
+        </is>
+      </c>
+      <c r="AC84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -7676,7 +8939,22 @@
       <c r="Y85" t="n">
         <v>1</v>
       </c>
-      <c r="Z85" t="inlineStr"/>
+      <c r="Z85" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_155/</t>
+        </is>
+      </c>
+      <c r="AA85" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_155/</t>
+        </is>
+      </c>
+      <c r="AB85" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_155/</t>
+        </is>
+      </c>
+      <c r="AC85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -7750,7 +9028,22 @@
       <c r="Y86" t="n">
         <v>1</v>
       </c>
-      <c r="Z86" t="inlineStr"/>
+      <c r="Z86" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_278/</t>
+        </is>
+      </c>
+      <c r="AA86" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_278/</t>
+        </is>
+      </c>
+      <c r="AB86" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_278/</t>
+        </is>
+      </c>
+      <c r="AC86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -7846,7 +9139,22 @@
       <c r="Y87" t="n">
         <v>1</v>
       </c>
-      <c r="Z87" t="inlineStr"/>
+      <c r="Z87" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_137/</t>
+        </is>
+      </c>
+      <c r="AA87" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_137/</t>
+        </is>
+      </c>
+      <c r="AB87" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_137/</t>
+        </is>
+      </c>
+      <c r="AC87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -7946,7 +9254,22 @@
       <c r="Y88" t="n">
         <v>1</v>
       </c>
-      <c r="Z88" t="inlineStr"/>
+      <c r="Z88" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_140/</t>
+        </is>
+      </c>
+      <c r="AA88" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_140/</t>
+        </is>
+      </c>
+      <c r="AB88" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_140/</t>
+        </is>
+      </c>
+      <c r="AC88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -8038,7 +9361,22 @@
       <c r="Y89" t="n">
         <v>3</v>
       </c>
-      <c r="Z89" t="inlineStr"/>
+      <c r="Z89" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_114/</t>
+        </is>
+      </c>
+      <c r="AA89" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_114/</t>
+        </is>
+      </c>
+      <c r="AB89" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_114/</t>
+        </is>
+      </c>
+      <c r="AC89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -8110,7 +9448,22 @@
       <c r="Y90" t="n">
         <v>1</v>
       </c>
-      <c r="Z90" t="inlineStr"/>
+      <c r="Z90" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_124/</t>
+        </is>
+      </c>
+      <c r="AA90" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_124/</t>
+        </is>
+      </c>
+      <c r="AB90" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_124/</t>
+        </is>
+      </c>
+      <c r="AC90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -8182,7 +9535,22 @@
       <c r="Y91" t="n">
         <v>1</v>
       </c>
-      <c r="Z91" t="inlineStr"/>
+      <c r="Z91" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_121/</t>
+        </is>
+      </c>
+      <c r="AA91" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_121/</t>
+        </is>
+      </c>
+      <c r="AB91" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_121/</t>
+        </is>
+      </c>
+      <c r="AC91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -8260,7 +9628,22 @@
       <c r="Y92" t="n">
         <v>1</v>
       </c>
-      <c r="Z92" t="inlineStr"/>
+      <c r="Z92" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_118/</t>
+        </is>
+      </c>
+      <c r="AA92" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_118/</t>
+        </is>
+      </c>
+      <c r="AB92" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_118/</t>
+        </is>
+      </c>
+      <c r="AC92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -8361,7 +9744,22 @@
       <c r="Y93" t="n">
         <v>2</v>
       </c>
-      <c r="Z93" t="inlineStr"/>
+      <c r="Z93" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_192/</t>
+        </is>
+      </c>
+      <c r="AA93" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_192/</t>
+        </is>
+      </c>
+      <c r="AB93" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_192/</t>
+        </is>
+      </c>
+      <c r="AC93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -8461,7 +9859,22 @@
       <c r="Y94" t="n">
         <v>1</v>
       </c>
-      <c r="Z94" t="inlineStr"/>
+      <c r="Z94" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_97/</t>
+        </is>
+      </c>
+      <c r="AA94" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_97/</t>
+        </is>
+      </c>
+      <c r="AB94" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_97/</t>
+        </is>
+      </c>
+      <c r="AC94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -8533,7 +9946,22 @@
       <c r="Y95" t="n">
         <v>1</v>
       </c>
-      <c r="Z95" t="inlineStr"/>
+      <c r="Z95" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_80/</t>
+        </is>
+      </c>
+      <c r="AA95" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_80/</t>
+        </is>
+      </c>
+      <c r="AB95" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_80/</t>
+        </is>
+      </c>
+      <c r="AC95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -8610,7 +10038,22 @@
       <c r="Y96" t="n">
         <v>1</v>
       </c>
-      <c r="Z96" t="inlineStr"/>
+      <c r="Z96" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_225/</t>
+        </is>
+      </c>
+      <c r="AA96" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_225/</t>
+        </is>
+      </c>
+      <c r="AB96" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_225/</t>
+        </is>
+      </c>
+      <c r="AC96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -8682,7 +10125,22 @@
       <c r="Y97" t="n">
         <v>1</v>
       </c>
-      <c r="Z97" t="inlineStr"/>
+      <c r="Z97" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_86/</t>
+        </is>
+      </c>
+      <c r="AA97" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_86/</t>
+        </is>
+      </c>
+      <c r="AB97" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_86/</t>
+        </is>
+      </c>
+      <c r="AC97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -8754,7 +10212,22 @@
       <c r="Y98" t="n">
         <v>1</v>
       </c>
-      <c r="Z98" t="inlineStr"/>
+      <c r="Z98" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_65/</t>
+        </is>
+      </c>
+      <c r="AA98" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_65/</t>
+        </is>
+      </c>
+      <c r="AB98" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_65/</t>
+        </is>
+      </c>
+      <c r="AC98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -8826,7 +10299,22 @@
       <c r="Y99" t="n">
         <v>1</v>
       </c>
-      <c r="Z99" t="inlineStr"/>
+      <c r="Z99" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_178/</t>
+        </is>
+      </c>
+      <c r="AA99" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_178/</t>
+        </is>
+      </c>
+      <c r="AB99" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_178/</t>
+        </is>
+      </c>
+      <c r="AC99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -8898,7 +10386,22 @@
       <c r="Y100" t="n">
         <v>1</v>
       </c>
-      <c r="Z100" t="inlineStr"/>
+      <c r="Z100" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_59/</t>
+        </is>
+      </c>
+      <c r="AA100" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_59/</t>
+        </is>
+      </c>
+      <c r="AB100" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_59/</t>
+        </is>
+      </c>
+      <c r="AC100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -8998,7 +10501,22 @@
       <c r="Y101" t="n">
         <v>1</v>
       </c>
-      <c r="Z101" t="inlineStr"/>
+      <c r="Z101" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_161/</t>
+        </is>
+      </c>
+      <c r="AA101" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_161/</t>
+        </is>
+      </c>
+      <c r="AB101" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_161/</t>
+        </is>
+      </c>
+      <c r="AC101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -9101,7 +10619,22 @@
       <c r="Y102" t="n">
         <v>1</v>
       </c>
-      <c r="Z102" t="inlineStr"/>
+      <c r="Z102" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_128/</t>
+        </is>
+      </c>
+      <c r="AA102" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_128/</t>
+        </is>
+      </c>
+      <c r="AB102" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_128/</t>
+        </is>
+      </c>
+      <c r="AC102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -9173,7 +10706,22 @@
       <c r="Y103" t="n">
         <v>1</v>
       </c>
-      <c r="Z103" t="inlineStr"/>
+      <c r="Z103" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_126/</t>
+        </is>
+      </c>
+      <c r="AA103" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_126/</t>
+        </is>
+      </c>
+      <c r="AB103" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_126/</t>
+        </is>
+      </c>
+      <c r="AC103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -9245,7 +10793,22 @@
       <c r="Y104" t="n">
         <v>1</v>
       </c>
-      <c r="Z104" t="inlineStr"/>
+      <c r="Z104" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_49/</t>
+        </is>
+      </c>
+      <c r="AA104" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_49/</t>
+        </is>
+      </c>
+      <c r="AB104" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_49/</t>
+        </is>
+      </c>
+      <c r="AC104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -9317,7 +10880,22 @@
       <c r="Y105" t="n">
         <v>2</v>
       </c>
-      <c r="Z105" t="inlineStr"/>
+      <c r="Z105" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_46/</t>
+        </is>
+      </c>
+      <c r="AA105" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_46/</t>
+        </is>
+      </c>
+      <c r="AB105" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_46/</t>
+        </is>
+      </c>
+      <c r="AC105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -9409,7 +10987,22 @@
       <c r="Y106" t="n">
         <v>2</v>
       </c>
-      <c r="Z106" t="inlineStr"/>
+      <c r="Z106" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_88/</t>
+        </is>
+      </c>
+      <c r="AA106" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_88/</t>
+        </is>
+      </c>
+      <c r="AB106" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_88/</t>
+        </is>
+      </c>
+      <c r="AC106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -9481,7 +11074,22 @@
       <c r="Y107" t="n">
         <v>1</v>
       </c>
-      <c r="Z107" t="inlineStr"/>
+      <c r="Z107" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_35/</t>
+        </is>
+      </c>
+      <c r="AA107" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_35/</t>
+        </is>
+      </c>
+      <c r="AB107" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_35/</t>
+        </is>
+      </c>
+      <c r="AC107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -9573,7 +11181,22 @@
       <c r="Y108" t="n">
         <v>1</v>
       </c>
-      <c r="Z108" t="inlineStr"/>
+      <c r="Z108" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2023_11/</t>
+        </is>
+      </c>
+      <c r="AA108" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2023_11/</t>
+        </is>
+      </c>
+      <c r="AB108" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2023_11/</t>
+        </is>
+      </c>
+      <c r="AC108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -9645,7 +11268,22 @@
       <c r="Y109" t="n">
         <v>1</v>
       </c>
-      <c r="Z109" t="inlineStr"/>
+      <c r="Z109" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_432/</t>
+        </is>
+      </c>
+      <c r="AA109" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_432/</t>
+        </is>
+      </c>
+      <c r="AB109" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_432/</t>
+        </is>
+      </c>
+      <c r="AC109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -9737,7 +11375,22 @@
       <c r="Y110" t="n">
         <v>5</v>
       </c>
-      <c r="Z110" t="inlineStr"/>
+      <c r="Z110" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_435/</t>
+        </is>
+      </c>
+      <c r="AA110" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_435/</t>
+        </is>
+      </c>
+      <c r="AB110" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_435/</t>
+        </is>
+      </c>
+      <c r="AC110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -9809,7 +11462,22 @@
       <c r="Y111" t="n">
         <v>1</v>
       </c>
-      <c r="Z111" t="inlineStr"/>
+      <c r="Z111" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_425/</t>
+        </is>
+      </c>
+      <c r="AA111" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_425/</t>
+        </is>
+      </c>
+      <c r="AB111" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_425/</t>
+        </is>
+      </c>
+      <c r="AC111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -9883,7 +11551,22 @@
       <c r="Y112" t="n">
         <v>1</v>
       </c>
-      <c r="Z112" t="inlineStr"/>
+      <c r="Z112" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_418/</t>
+        </is>
+      </c>
+      <c r="AA112" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_418/</t>
+        </is>
+      </c>
+      <c r="AB112" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_418/</t>
+        </is>
+      </c>
+      <c r="AC112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -9957,7 +11640,22 @@
       <c r="Y113" t="n">
         <v>2</v>
       </c>
-      <c r="Z113" t="inlineStr"/>
+      <c r="Z113" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_408/</t>
+        </is>
+      </c>
+      <c r="AA113" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_408/</t>
+        </is>
+      </c>
+      <c r="AB113" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_408/</t>
+        </is>
+      </c>
+      <c r="AC113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -10031,7 +11729,22 @@
       <c r="Y114" t="n">
         <v>1</v>
       </c>
-      <c r="Z114" t="inlineStr"/>
+      <c r="Z114" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_422/</t>
+        </is>
+      </c>
+      <c r="AA114" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_422/</t>
+        </is>
+      </c>
+      <c r="AB114" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_422/</t>
+        </is>
+      </c>
+      <c r="AC114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -10123,7 +11836,22 @@
       <c r="Y115" t="n">
         <v>1</v>
       </c>
-      <c r="Z115" t="inlineStr"/>
+      <c r="Z115" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_414/</t>
+        </is>
+      </c>
+      <c r="AA115" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_414/</t>
+        </is>
+      </c>
+      <c r="AB115" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_414/</t>
+        </is>
+      </c>
+      <c r="AC115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -10195,7 +11923,22 @@
       <c r="Y116" t="n">
         <v>1</v>
       </c>
-      <c r="Z116" t="inlineStr"/>
+      <c r="Z116" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_401/</t>
+        </is>
+      </c>
+      <c r="AA116" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_401/</t>
+        </is>
+      </c>
+      <c r="AB116" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_401/</t>
+        </is>
+      </c>
+      <c r="AC116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -10269,7 +12012,22 @@
       <c r="Y117" t="n">
         <v>1</v>
       </c>
-      <c r="Z117" t="inlineStr"/>
+      <c r="Z117" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_393/</t>
+        </is>
+      </c>
+      <c r="AA117" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_393/</t>
+        </is>
+      </c>
+      <c r="AB117" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_393/</t>
+        </is>
+      </c>
+      <c r="AC117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -10343,7 +12101,22 @@
       <c r="Y118" t="n">
         <v>1</v>
       </c>
-      <c r="Z118" t="inlineStr"/>
+      <c r="Z118" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_762/</t>
+        </is>
+      </c>
+      <c r="AA118" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_762/</t>
+        </is>
+      </c>
+      <c r="AB118" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_762/</t>
+        </is>
+      </c>
+      <c r="AC118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -10415,7 +12188,22 @@
       <c r="Y119" t="n">
         <v>1</v>
       </c>
-      <c r="Z119" t="inlineStr"/>
+      <c r="Z119" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_697/</t>
+        </is>
+      </c>
+      <c r="AA119" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_697/</t>
+        </is>
+      </c>
+      <c r="AB119" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_697/</t>
+        </is>
+      </c>
+      <c r="AC119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -10487,7 +12275,22 @@
       <c r="Y120" t="n">
         <v>1</v>
       </c>
-      <c r="Z120" t="inlineStr"/>
+      <c r="Z120" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_395/</t>
+        </is>
+      </c>
+      <c r="AA120" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_395/</t>
+        </is>
+      </c>
+      <c r="AB120" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_395/</t>
+        </is>
+      </c>
+      <c r="AC120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -10559,7 +12362,22 @@
       <c r="Y121" t="n">
         <v>1</v>
       </c>
-      <c r="Z121" t="inlineStr"/>
+      <c r="Z121" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_391/</t>
+        </is>
+      </c>
+      <c r="AA121" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_391/</t>
+        </is>
+      </c>
+      <c r="AB121" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_391/</t>
+        </is>
+      </c>
+      <c r="AC121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -10631,7 +12449,22 @@
       <c r="Y122" t="n">
         <v>2</v>
       </c>
-      <c r="Z122" t="inlineStr"/>
+      <c r="Z122" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_384/</t>
+        </is>
+      </c>
+      <c r="AA122" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_384/</t>
+        </is>
+      </c>
+      <c r="AB122" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_384/</t>
+        </is>
+      </c>
+      <c r="AC122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -10703,7 +12536,22 @@
       <c r="Y123" t="n">
         <v>2</v>
       </c>
-      <c r="Z123" t="inlineStr"/>
+      <c r="Z123" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_377/</t>
+        </is>
+      </c>
+      <c r="AA123" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_377/</t>
+        </is>
+      </c>
+      <c r="AB123" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_377/</t>
+        </is>
+      </c>
+      <c r="AC123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -10798,7 +12646,22 @@
       <c r="Y124" t="n">
         <v>1</v>
       </c>
-      <c r="Z124" t="inlineStr"/>
+      <c r="Z124" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_368/</t>
+        </is>
+      </c>
+      <c r="AA124" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_368/</t>
+        </is>
+      </c>
+      <c r="AB124" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_368/</t>
+        </is>
+      </c>
+      <c r="AC124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -10890,7 +12753,22 @@
       <c r="Y125" t="n">
         <v>1</v>
       </c>
-      <c r="Z125" t="inlineStr"/>
+      <c r="Z125" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_721/</t>
+        </is>
+      </c>
+      <c r="AA125" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_721/</t>
+        </is>
+      </c>
+      <c r="AB125" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_721/</t>
+        </is>
+      </c>
+      <c r="AC125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -10962,7 +12840,22 @@
       <c r="Y126" t="n">
         <v>3</v>
       </c>
-      <c r="Z126" t="inlineStr"/>
+      <c r="Z126" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_359/</t>
+        </is>
+      </c>
+      <c r="AA126" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_359/</t>
+        </is>
+      </c>
+      <c r="AB126" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_359/</t>
+        </is>
+      </c>
+      <c r="AC126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -11034,7 +12927,22 @@
       <c r="Y127" t="n">
         <v>1</v>
       </c>
-      <c r="Z127" t="inlineStr"/>
+      <c r="Z127" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_350/</t>
+        </is>
+      </c>
+      <c r="AA127" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_350/</t>
+        </is>
+      </c>
+      <c r="AB127" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_350/</t>
+        </is>
+      </c>
+      <c r="AC127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -11106,7 +13014,22 @@
       <c r="Y128" t="n">
         <v>1</v>
       </c>
-      <c r="Z128" t="inlineStr"/>
+      <c r="Z128" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_298/</t>
+        </is>
+      </c>
+      <c r="AA128" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_298/</t>
+        </is>
+      </c>
+      <c r="AB128" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_298/</t>
+        </is>
+      </c>
+      <c r="AC128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -11178,7 +13101,22 @@
       <c r="Y129" t="n">
         <v>1</v>
       </c>
-      <c r="Z129" t="inlineStr"/>
+      <c r="Z129" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_546/</t>
+        </is>
+      </c>
+      <c r="AA129" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_546/</t>
+        </is>
+      </c>
+      <c r="AB129" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_546/</t>
+        </is>
+      </c>
+      <c r="AC129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -11250,7 +13188,22 @@
       <c r="Y130" t="n">
         <v>4</v>
       </c>
-      <c r="Z130" t="inlineStr"/>
+      <c r="Z130" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_545/</t>
+        </is>
+      </c>
+      <c r="AA130" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_545/</t>
+        </is>
+      </c>
+      <c r="AB130" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_545/</t>
+        </is>
+      </c>
+      <c r="AC130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -11322,7 +13275,22 @@
       <c r="Y131" t="n">
         <v>1</v>
       </c>
-      <c r="Z131" t="inlineStr"/>
+      <c r="Z131" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_541/</t>
+        </is>
+      </c>
+      <c r="AA131" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_541/</t>
+        </is>
+      </c>
+      <c r="AB131" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_541/</t>
+        </is>
+      </c>
+      <c r="AC131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -11414,7 +13382,22 @@
       <c r="Y132" t="n">
         <v>1</v>
       </c>
-      <c r="Z132" t="inlineStr"/>
+      <c r="Z132" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_540/</t>
+        </is>
+      </c>
+      <c r="AA132" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_540/</t>
+        </is>
+      </c>
+      <c r="AB132" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_540/</t>
+        </is>
+      </c>
+      <c r="AC132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -11486,7 +13469,22 @@
       <c r="Y133" t="n">
         <v>1</v>
       </c>
-      <c r="Z133" t="inlineStr"/>
+      <c r="Z133" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_321/</t>
+        </is>
+      </c>
+      <c r="AA133" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_321/</t>
+        </is>
+      </c>
+      <c r="AB133" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_321/</t>
+        </is>
+      </c>
+      <c r="AC133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -11582,7 +13580,22 @@
       <c r="Y134" t="n">
         <v>1</v>
       </c>
-      <c r="Z134" t="inlineStr"/>
+      <c r="Z134" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_319/</t>
+        </is>
+      </c>
+      <c r="AA134" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_319/</t>
+        </is>
+      </c>
+      <c r="AB134" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_319/</t>
+        </is>
+      </c>
+      <c r="AC134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -11654,7 +13667,22 @@
       <c r="Y135" t="n">
         <v>1</v>
       </c>
-      <c r="Z135" t="inlineStr"/>
+      <c r="Z135" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_316/</t>
+        </is>
+      </c>
+      <c r="AA135" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_316/</t>
+        </is>
+      </c>
+      <c r="AB135" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_316/</t>
+        </is>
+      </c>
+      <c r="AC135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -11726,7 +13754,22 @@
       <c r="Y136" t="n">
         <v>1</v>
       </c>
-      <c r="Z136" t="inlineStr"/>
+      <c r="Z136" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_311/</t>
+        </is>
+      </c>
+      <c r="AA136" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_311/</t>
+        </is>
+      </c>
+      <c r="AB136" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_311/</t>
+        </is>
+      </c>
+      <c r="AC136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -11826,7 +13869,22 @@
       <c r="Y137" t="n">
         <v>2</v>
       </c>
-      <c r="Z137" t="inlineStr"/>
+      <c r="Z137" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_289/</t>
+        </is>
+      </c>
+      <c r="AA137" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_289/</t>
+        </is>
+      </c>
+      <c r="AB137" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_289/</t>
+        </is>
+      </c>
+      <c r="AC137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -11898,7 +13956,22 @@
       <c r="Y138" t="n">
         <v>3</v>
       </c>
-      <c r="Z138" t="inlineStr"/>
+      <c r="Z138" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_286/</t>
+        </is>
+      </c>
+      <c r="AA138" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_286/</t>
+        </is>
+      </c>
+      <c r="AB138" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_286/</t>
+        </is>
+      </c>
+      <c r="AC138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -11970,7 +14043,22 @@
       <c r="Y139" t="n">
         <v>3</v>
       </c>
-      <c r="Z139" t="inlineStr"/>
+      <c r="Z139" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_282/</t>
+        </is>
+      </c>
+      <c r="AA139" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_282/</t>
+        </is>
+      </c>
+      <c r="AB139" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_282/</t>
+        </is>
+      </c>
+      <c r="AC139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -12042,7 +14130,22 @@
       <c r="Y140" t="n">
         <v>3</v>
       </c>
-      <c r="Z140" t="inlineStr"/>
+      <c r="Z140" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_190/</t>
+        </is>
+      </c>
+      <c r="AA140" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_190/</t>
+        </is>
+      </c>
+      <c r="AB140" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_190/</t>
+        </is>
+      </c>
+      <c r="AC140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -12142,7 +14245,22 @@
       <c r="Y141" t="n">
         <v>2</v>
       </c>
-      <c r="Z141" t="inlineStr"/>
+      <c r="Z141" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_170/</t>
+        </is>
+      </c>
+      <c r="AA141" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_170/</t>
+        </is>
+      </c>
+      <c r="AB141" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_170/</t>
+        </is>
+      </c>
+      <c r="AC141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -12238,7 +14356,22 @@
       <c r="Y142" t="n">
         <v>12</v>
       </c>
-      <c r="Z142" t="inlineStr"/>
+      <c r="Z142" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_167/</t>
+        </is>
+      </c>
+      <c r="AA142" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_167/</t>
+        </is>
+      </c>
+      <c r="AB142" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_167/</t>
+        </is>
+      </c>
+      <c r="AC142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -12310,7 +14443,22 @@
       <c r="Y143" t="n">
         <v>1</v>
       </c>
-      <c r="Z143" t="inlineStr"/>
+      <c r="Z143" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_245/</t>
+        </is>
+      </c>
+      <c r="AA143" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_245/</t>
+        </is>
+      </c>
+      <c r="AB143" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_245/</t>
+        </is>
+      </c>
+      <c r="AC143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -12382,7 +14530,22 @@
       <c r="Y144" t="n">
         <v>1</v>
       </c>
-      <c r="Z144" t="inlineStr"/>
+      <c r="Z144" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_209/</t>
+        </is>
+      </c>
+      <c r="AA144" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_209/</t>
+        </is>
+      </c>
+      <c r="AB144" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_209/</t>
+        </is>
+      </c>
+      <c r="AC144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -12474,7 +14637,22 @@
       <c r="Y145" t="n">
         <v>1</v>
       </c>
-      <c r="Z145" t="inlineStr"/>
+      <c r="Z145" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_145/</t>
+        </is>
+      </c>
+      <c r="AA145" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_145/</t>
+        </is>
+      </c>
+      <c r="AB145" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_145/</t>
+        </is>
+      </c>
+      <c r="AC145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -12546,7 +14724,22 @@
       <c r="Y146" t="n">
         <v>1</v>
       </c>
-      <c r="Z146" t="inlineStr"/>
+      <c r="Z146" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_141/</t>
+        </is>
+      </c>
+      <c r="AA146" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_141/</t>
+        </is>
+      </c>
+      <c r="AB146" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_141/</t>
+        </is>
+      </c>
+      <c r="AC146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -12638,7 +14831,22 @@
       <c r="Y147" t="n">
         <v>4</v>
       </c>
-      <c r="Z147" t="inlineStr"/>
+      <c r="Z147" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_131/</t>
+        </is>
+      </c>
+      <c r="AA147" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_131/</t>
+        </is>
+      </c>
+      <c r="AB147" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_131/</t>
+        </is>
+      </c>
+      <c r="AC147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -12710,7 +14918,22 @@
       <c r="Y148" t="n">
         <v>1</v>
       </c>
-      <c r="Z148" t="inlineStr"/>
+      <c r="Z148" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_658/</t>
+        </is>
+      </c>
+      <c r="AA148" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_658/</t>
+        </is>
+      </c>
+      <c r="AB148" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_658/</t>
+        </is>
+      </c>
+      <c r="AC148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -12782,7 +15005,22 @@
       <c r="Y149" t="n">
         <v>1</v>
       </c>
-      <c r="Z149" t="inlineStr"/>
+      <c r="Z149" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_656/</t>
+        </is>
+      </c>
+      <c r="AA149" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_656/</t>
+        </is>
+      </c>
+      <c r="AB149" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_656/</t>
+        </is>
+      </c>
+      <c r="AC149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -12854,7 +15092,22 @@
       <c r="Y150" t="n">
         <v>1</v>
       </c>
-      <c r="Z150" t="inlineStr"/>
+      <c r="Z150" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_651/</t>
+        </is>
+      </c>
+      <c r="AA150" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_651/</t>
+        </is>
+      </c>
+      <c r="AB150" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_651/</t>
+        </is>
+      </c>
+      <c r="AC150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -12926,7 +15179,22 @@
       <c r="Y151" t="n">
         <v>1</v>
       </c>
-      <c r="Z151" t="inlineStr"/>
+      <c r="Z151" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_115/</t>
+        </is>
+      </c>
+      <c r="AA151" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_115/</t>
+        </is>
+      </c>
+      <c r="AB151" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_115/</t>
+        </is>
+      </c>
+      <c r="AC151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -12998,7 +15266,22 @@
       <c r="Y152" t="n">
         <v>1</v>
       </c>
-      <c r="Z152" t="inlineStr"/>
+      <c r="Z152" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_99/</t>
+        </is>
+      </c>
+      <c r="AA152" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_99/</t>
+        </is>
+      </c>
+      <c r="AB152" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_99/</t>
+        </is>
+      </c>
+      <c r="AC152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -13070,7 +15353,22 @@
       <c r="Y153" t="n">
         <v>2</v>
       </c>
-      <c r="Z153" t="inlineStr"/>
+      <c r="Z153" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_96/</t>
+        </is>
+      </c>
+      <c r="AA153" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_96/</t>
+        </is>
+      </c>
+      <c r="AB153" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_96/</t>
+        </is>
+      </c>
+      <c r="AC153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -13174,7 +15472,22 @@
       <c r="Y154" t="n">
         <v>5</v>
       </c>
-      <c r="Z154" t="inlineStr"/>
+      <c r="Z154" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_111/</t>
+        </is>
+      </c>
+      <c r="AA154" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_111/</t>
+        </is>
+      </c>
+      <c r="AB154" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_111/</t>
+        </is>
+      </c>
+      <c r="AC154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -13246,7 +15559,22 @@
       <c r="Y155" t="n">
         <v>2</v>
       </c>
-      <c r="Z155" t="inlineStr"/>
+      <c r="Z155" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_135/</t>
+        </is>
+      </c>
+      <c r="AA155" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_135/</t>
+        </is>
+      </c>
+      <c r="AB155" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_135/</t>
+        </is>
+      </c>
+      <c r="AC155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -13318,7 +15646,22 @@
       <c r="Y156" t="n">
         <v>1</v>
       </c>
-      <c r="Z156" t="inlineStr"/>
+      <c r="Z156" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_88/</t>
+        </is>
+      </c>
+      <c r="AA156" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_88/</t>
+        </is>
+      </c>
+      <c r="AB156" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_88/</t>
+        </is>
+      </c>
+      <c r="AC156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -13390,7 +15733,22 @@
       <c r="Y157" t="n">
         <v>1</v>
       </c>
-      <c r="Z157" t="inlineStr"/>
+      <c r="Z157" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_85/</t>
+        </is>
+      </c>
+      <c r="AA157" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_85/</t>
+        </is>
+      </c>
+      <c r="AB157" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_85/</t>
+        </is>
+      </c>
+      <c r="AC157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -13482,7 +15840,22 @@
       <c r="Y158" t="n">
         <v>4</v>
       </c>
-      <c r="Z158" t="inlineStr"/>
+      <c r="Z158" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_82/</t>
+        </is>
+      </c>
+      <c r="AA158" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_82/</t>
+        </is>
+      </c>
+      <c r="AB158" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_82/</t>
+        </is>
+      </c>
+      <c r="AC158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -13555,7 +15928,22 @@
       <c r="Y159" t="n">
         <v>1</v>
       </c>
-      <c r="Z159" t="inlineStr"/>
+      <c r="Z159" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_75/</t>
+        </is>
+      </c>
+      <c r="AA159" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_75/</t>
+        </is>
+      </c>
+      <c r="AB159" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_75/</t>
+        </is>
+      </c>
+      <c r="AC159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -13627,7 +16015,22 @@
       <c r="Y160" t="n">
         <v>1</v>
       </c>
-      <c r="Z160" t="inlineStr"/>
+      <c r="Z160" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_62/</t>
+        </is>
+      </c>
+      <c r="AA160" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_62/</t>
+        </is>
+      </c>
+      <c r="AB160" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_62/</t>
+        </is>
+      </c>
+      <c r="AC160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -13699,7 +16102,22 @@
       <c r="Y161" t="n">
         <v>2</v>
       </c>
-      <c r="Z161" t="inlineStr"/>
+      <c r="Z161" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_42/</t>
+        </is>
+      </c>
+      <c r="AA161" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_42/</t>
+        </is>
+      </c>
+      <c r="AB161" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_42/</t>
+        </is>
+      </c>
+      <c r="AC161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -13772,7 +16190,22 @@
       <c r="Y162" t="n">
         <v>1</v>
       </c>
-      <c r="Z162" t="inlineStr"/>
+      <c r="Z162" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_34/</t>
+        </is>
+      </c>
+      <c r="AA162" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_34/</t>
+        </is>
+      </c>
+      <c r="AB162" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_34/</t>
+        </is>
+      </c>
+      <c r="AC162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -13864,7 +16297,22 @@
       <c r="Y163" t="n">
         <v>1</v>
       </c>
-      <c r="Z163" t="inlineStr"/>
+      <c r="Z163" s="2" t="inlineStr">
+        <is>
+          <t>pdfs/SWD_2022_30/</t>
+        </is>
+      </c>
+      <c r="AA163" s="2" t="inlineStr">
+        <is>
+          <t>md/SWD_2022_30/</t>
+        </is>
+      </c>
+      <c r="AB163" s="2" t="inlineStr">
+        <is>
+          <t>docx/SWD_2022_30/</t>
+        </is>
+      </c>
+      <c r="AC163" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="3">
@@ -13881,233 +16329,719 @@
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A9" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A13" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A14" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A15" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A16" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A17" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A18" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A19" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A20" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A21" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A22" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A23" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A24" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A25" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A26" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A27" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A28" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A29" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A30" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A31" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A32" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K32" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A33" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K33" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A34" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A35" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A36" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A37" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A38" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A39" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A40" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A41" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K41" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A42" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K42" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A43" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A44" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K44" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A45" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A46" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K46" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A47" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A48" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K48" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A49" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A50" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K50" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A51" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K51" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A52" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K52" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A53" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K53" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A54" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A55" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A56" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K56" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A57" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A58" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A59" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K59" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A60" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K60" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A61" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A62" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A63" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K63" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A64" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A65" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A66" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K66" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A67" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K67" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A68" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K68" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A69" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A70" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K70" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A71" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K71" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A72" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A73" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K73" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A74" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A75" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A76" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A77" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A78" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A79" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K79" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A80" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A81" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K81" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A82" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K82" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A83" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A84" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A85" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K85" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A86" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A87" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K87" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A88" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K88" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A89" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K89" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A90" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A91" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A92" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A93" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K93" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A94" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K94" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A95" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A96" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A97" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A98" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A99" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A100" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A101" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K101" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A102" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K102" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A103" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A104" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A105" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A106" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K106" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A107" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A108" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K108" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A109" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A110" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K110" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A111" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A112" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A113" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A114" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A115" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K115" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A116" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A117" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A118" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A119" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A120" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A121" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A122" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A123" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A124" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K124" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A125" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K125" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A126" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A127" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A128" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A129" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A130" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A131" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A132" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K132" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A133" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A134" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K134" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A135" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A136" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A137" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K137" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A138" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A139" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A140" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A141" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K141" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A142" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K142" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A143" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A144" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A145" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K145" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A146" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A147" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K147" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A148" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A149" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A150" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A151" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A152" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A153" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A154" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K154" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A155" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A156" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A157" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A158" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K158" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A159" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A160" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A161" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A162" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A163" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K163" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z2" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA2" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB2" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z3" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA3" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB3" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z4" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA4" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB4" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z5" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA5" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB5" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z6" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA6" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB6" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z7" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA7" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB7" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z8" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA8" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB8" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A9" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z9" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA9" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB9" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z10" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA10" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB10" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z11" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA11" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB11" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z12" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA12" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB12" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A13" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z13" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA13" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB13" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A14" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z14" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA14" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB14" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A15" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z15" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA15" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB15" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A16" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z16" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA16" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB16" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A17" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z17" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA17" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB17" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A18" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z18" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA18" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB18" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A19" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z19" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA19" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB19" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A20" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z20" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA20" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB20" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A21" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z21" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA21" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB21" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A22" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z22" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA22" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB22" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A23" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z23" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA23" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB23" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A24" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z24" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA24" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB24" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A25" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z25" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA25" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB25" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A26" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z26" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA26" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB26" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A27" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z27" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA27" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB27" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A28" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z28" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA28" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB28" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A29" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z29" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA29" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB29" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A30" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z30" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA30" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB30" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A31" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z31" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA31" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB31" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A32" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K32" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z32" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA32" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB32" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A33" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K33" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z33" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA33" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB33" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A34" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z34" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA34" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB34" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A35" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z35" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA35" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB35" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A36" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z36" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA36" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB36" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A37" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z37" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA37" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB37" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A38" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z38" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA38" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB38" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A39" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z39" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA39" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB39" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A40" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z40" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA40" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB40" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A41" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K41" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z41" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA41" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB41" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A42" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K42" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z42" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA42" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB42" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A43" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z43" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA43" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB43" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A44" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K44" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z44" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA44" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB44" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A45" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z45" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA45" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB45" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A46" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K46" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z46" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA46" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB46" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A47" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z47" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA47" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB47" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A48" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K48" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z48" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA48" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB48" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A49" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z49" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA49" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB49" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A50" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K50" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z50" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA50" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB50" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A51" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K51" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z51" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA51" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB51" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A52" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K52" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z52" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA52" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB52" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A53" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K53" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z53" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA53" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB53" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A54" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z54" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA54" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB54" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A55" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z55" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA55" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB55" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A56" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K56" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z56" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA56" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB56" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A57" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z57" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA57" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB57" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A58" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z58" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA58" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB58" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A59" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K59" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z59" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA59" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB59" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A60" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K60" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z60" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA60" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB60" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A61" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z61" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA61" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB61" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A62" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z62" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA62" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB62" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A63" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K63" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z63" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA63" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB63" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A64" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z64" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA64" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB64" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A65" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z65" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA65" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB65" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A66" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K66" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z66" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA66" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB66" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A67" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K67" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z67" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA67" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB67" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A68" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K68" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z68" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA68" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB68" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A69" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z69" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA69" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB69" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A70" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K70" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z70" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA70" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB70" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A71" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K71" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z71" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA71" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB71" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A72" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z72" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA72" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB72" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A73" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K73" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z73" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA73" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB73" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A74" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z74" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA74" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB74" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A75" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z75" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA75" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB75" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A76" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z76" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA76" r:id="rId339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB76" r:id="rId340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A77" r:id="rId341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z77" r:id="rId342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA77" r:id="rId343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB77" r:id="rId344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A78" r:id="rId345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z78" r:id="rId346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA78" r:id="rId347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB78" r:id="rId348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A79" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K79" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z79" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA79" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB79" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A80" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z80" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA80" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB80" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A81" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K81" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z81" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA81" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB81" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A82" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K82" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z82" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA82" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB82" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A83" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z83" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA83" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB83" r:id="rId371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A84" r:id="rId372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z84" r:id="rId373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA84" r:id="rId374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB84" r:id="rId375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A85" r:id="rId376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K85" r:id="rId377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z85" r:id="rId378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA85" r:id="rId379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB85" r:id="rId380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A86" r:id="rId381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z86" r:id="rId382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA86" r:id="rId383"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB86" r:id="rId384"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A87" r:id="rId385"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K87" r:id="rId386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z87" r:id="rId387"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA87" r:id="rId388"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB87" r:id="rId389"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A88" r:id="rId390"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K88" r:id="rId391"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z88" r:id="rId392"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA88" r:id="rId393"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB88" r:id="rId394"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A89" r:id="rId395"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K89" r:id="rId396"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z89" r:id="rId397"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA89" r:id="rId398"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB89" r:id="rId399"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A90" r:id="rId400"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z90" r:id="rId401"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA90" r:id="rId402"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB90" r:id="rId403"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A91" r:id="rId404"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z91" r:id="rId405"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA91" r:id="rId406"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB91" r:id="rId407"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A92" r:id="rId408"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z92" r:id="rId409"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA92" r:id="rId410"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB92" r:id="rId411"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A93" r:id="rId412"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K93" r:id="rId413"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z93" r:id="rId414"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA93" r:id="rId415"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB93" r:id="rId416"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A94" r:id="rId417"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K94" r:id="rId418"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z94" r:id="rId419"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA94" r:id="rId420"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB94" r:id="rId421"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A95" r:id="rId422"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z95" r:id="rId423"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA95" r:id="rId424"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB95" r:id="rId425"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A96" r:id="rId426"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z96" r:id="rId427"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA96" r:id="rId428"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB96" r:id="rId429"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A97" r:id="rId430"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z97" r:id="rId431"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA97" r:id="rId432"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB97" r:id="rId433"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A98" r:id="rId434"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z98" r:id="rId435"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA98" r:id="rId436"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB98" r:id="rId437"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A99" r:id="rId438"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z99" r:id="rId439"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA99" r:id="rId440"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB99" r:id="rId441"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A100" r:id="rId442"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z100" r:id="rId443"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA100" r:id="rId444"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB100" r:id="rId445"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A101" r:id="rId446"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K101" r:id="rId447"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z101" r:id="rId448"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA101" r:id="rId449"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB101" r:id="rId450"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A102" r:id="rId451"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K102" r:id="rId452"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z102" r:id="rId453"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA102" r:id="rId454"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB102" r:id="rId455"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A103" r:id="rId456"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z103" r:id="rId457"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA103" r:id="rId458"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB103" r:id="rId459"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A104" r:id="rId460"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z104" r:id="rId461"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA104" r:id="rId462"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB104" r:id="rId463"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A105" r:id="rId464"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z105" r:id="rId465"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA105" r:id="rId466"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB105" r:id="rId467"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A106" r:id="rId468"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K106" r:id="rId469"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z106" r:id="rId470"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA106" r:id="rId471"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB106" r:id="rId472"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A107" r:id="rId473"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z107" r:id="rId474"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA107" r:id="rId475"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB107" r:id="rId476"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A108" r:id="rId477"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K108" r:id="rId478"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z108" r:id="rId479"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA108" r:id="rId480"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB108" r:id="rId481"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A109" r:id="rId482"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z109" r:id="rId483"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA109" r:id="rId484"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB109" r:id="rId485"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A110" r:id="rId486"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K110" r:id="rId487"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z110" r:id="rId488"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA110" r:id="rId489"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB110" r:id="rId490"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A111" r:id="rId491"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z111" r:id="rId492"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA111" r:id="rId493"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB111" r:id="rId494"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A112" r:id="rId495"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z112" r:id="rId496"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA112" r:id="rId497"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB112" r:id="rId498"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A113" r:id="rId499"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z113" r:id="rId500"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA113" r:id="rId501"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB113" r:id="rId502"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A114" r:id="rId503"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z114" r:id="rId504"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA114" r:id="rId505"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB114" r:id="rId506"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A115" r:id="rId507"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K115" r:id="rId508"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z115" r:id="rId509"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA115" r:id="rId510"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB115" r:id="rId511"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A116" r:id="rId512"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z116" r:id="rId513"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA116" r:id="rId514"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB116" r:id="rId515"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A117" r:id="rId516"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z117" r:id="rId517"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA117" r:id="rId518"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB117" r:id="rId519"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A118" r:id="rId520"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z118" r:id="rId521"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA118" r:id="rId522"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB118" r:id="rId523"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A119" r:id="rId524"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z119" r:id="rId525"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA119" r:id="rId526"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB119" r:id="rId527"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A120" r:id="rId528"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z120" r:id="rId529"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA120" r:id="rId530"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB120" r:id="rId531"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A121" r:id="rId532"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z121" r:id="rId533"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA121" r:id="rId534"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB121" r:id="rId535"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A122" r:id="rId536"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z122" r:id="rId537"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA122" r:id="rId538"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB122" r:id="rId539"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A123" r:id="rId540"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z123" r:id="rId541"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA123" r:id="rId542"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB123" r:id="rId543"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A124" r:id="rId544"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K124" r:id="rId545"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z124" r:id="rId546"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA124" r:id="rId547"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB124" r:id="rId548"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A125" r:id="rId549"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K125" r:id="rId550"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z125" r:id="rId551"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA125" r:id="rId552"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB125" r:id="rId553"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A126" r:id="rId554"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z126" r:id="rId555"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA126" r:id="rId556"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB126" r:id="rId557"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A127" r:id="rId558"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z127" r:id="rId559"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA127" r:id="rId560"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB127" r:id="rId561"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A128" r:id="rId562"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z128" r:id="rId563"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA128" r:id="rId564"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB128" r:id="rId565"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A129" r:id="rId566"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z129" r:id="rId567"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA129" r:id="rId568"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB129" r:id="rId569"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A130" r:id="rId570"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z130" r:id="rId571"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA130" r:id="rId572"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB130" r:id="rId573"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A131" r:id="rId574"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z131" r:id="rId575"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA131" r:id="rId576"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB131" r:id="rId577"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A132" r:id="rId578"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K132" r:id="rId579"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z132" r:id="rId580"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA132" r:id="rId581"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB132" r:id="rId582"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A133" r:id="rId583"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z133" r:id="rId584"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA133" r:id="rId585"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB133" r:id="rId586"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A134" r:id="rId587"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K134" r:id="rId588"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z134" r:id="rId589"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA134" r:id="rId590"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB134" r:id="rId591"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A135" r:id="rId592"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z135" r:id="rId593"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA135" r:id="rId594"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB135" r:id="rId595"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A136" r:id="rId596"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z136" r:id="rId597"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA136" r:id="rId598"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB136" r:id="rId599"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A137" r:id="rId600"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K137" r:id="rId601"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z137" r:id="rId602"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA137" r:id="rId603"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB137" r:id="rId604"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A138" r:id="rId605"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z138" r:id="rId606"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA138" r:id="rId607"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB138" r:id="rId608"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A139" r:id="rId609"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z139" r:id="rId610"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA139" r:id="rId611"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB139" r:id="rId612"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A140" r:id="rId613"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z140" r:id="rId614"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA140" r:id="rId615"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB140" r:id="rId616"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A141" r:id="rId617"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K141" r:id="rId618"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z141" r:id="rId619"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA141" r:id="rId620"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB141" r:id="rId621"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A142" r:id="rId622"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K142" r:id="rId623"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z142" r:id="rId624"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA142" r:id="rId625"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB142" r:id="rId626"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A143" r:id="rId627"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z143" r:id="rId628"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA143" r:id="rId629"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB143" r:id="rId630"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A144" r:id="rId631"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z144" r:id="rId632"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA144" r:id="rId633"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB144" r:id="rId634"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A145" r:id="rId635"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K145" r:id="rId636"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z145" r:id="rId637"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA145" r:id="rId638"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB145" r:id="rId639"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A146" r:id="rId640"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z146" r:id="rId641"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA146" r:id="rId642"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB146" r:id="rId643"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A147" r:id="rId644"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K147" r:id="rId645"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z147" r:id="rId646"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA147" r:id="rId647"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB147" r:id="rId648"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A148" r:id="rId649"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z148" r:id="rId650"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA148" r:id="rId651"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB148" r:id="rId652"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A149" r:id="rId653"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z149" r:id="rId654"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA149" r:id="rId655"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB149" r:id="rId656"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A150" r:id="rId657"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z150" r:id="rId658"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA150" r:id="rId659"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB150" r:id="rId660"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A151" r:id="rId661"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z151" r:id="rId662"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA151" r:id="rId663"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB151" r:id="rId664"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A152" r:id="rId665"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z152" r:id="rId666"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA152" r:id="rId667"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB152" r:id="rId668"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A153" r:id="rId669"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z153" r:id="rId670"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA153" r:id="rId671"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB153" r:id="rId672"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A154" r:id="rId673"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K154" r:id="rId674"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z154" r:id="rId675"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA154" r:id="rId676"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB154" r:id="rId677"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A155" r:id="rId678"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z155" r:id="rId679"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA155" r:id="rId680"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB155" r:id="rId681"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A156" r:id="rId682"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z156" r:id="rId683"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA156" r:id="rId684"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB156" r:id="rId685"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A157" r:id="rId686"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z157" r:id="rId687"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA157" r:id="rId688"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB157" r:id="rId689"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A158" r:id="rId690"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K158" r:id="rId691"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z158" r:id="rId692"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA158" r:id="rId693"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB158" r:id="rId694"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A159" r:id="rId695"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z159" r:id="rId696"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA159" r:id="rId697"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB159" r:id="rId698"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A160" r:id="rId699"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z160" r:id="rId700"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA160" r:id="rId701"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB160" r:id="rId702"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A161" r:id="rId703"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z161" r:id="rId704"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA161" r:id="rId705"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB161" r:id="rId706"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A162" r:id="rId707"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z162" r:id="rId708"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA162" r:id="rId709"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB162" r:id="rId710"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A163" r:id="rId711"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K163" r:id="rId712"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z163" r:id="rId713"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA163" r:id="rId714"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB163" r:id="rId715"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>